<commit_message>
description of Energy datasets
</commit_message>
<xml_diff>
--- a/datasets/Energy/Details of Dataset/Details of Datasets.xlsx
+++ b/datasets/Energy/Details of Dataset/Details of Datasets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HiWi\tabbank\datasets\Energy\Details of Dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2534420C-D301-4998-8BAD-3C6673F0642E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84DF6950-24DA-4A5F-9BD0-D8DAB5BB9492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA6F8067-0B2C-427F-AF2F-C339AFBDD94F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="176">
   <si>
     <t>Link</t>
   </si>
@@ -217,15 +217,9 @@
     <t>19K</t>
   </si>
   <si>
-    <t>energydata_complete.csv</t>
-  </si>
-  <si>
     <t>The dataset contains data points collected from a Combined Cycle Power Plant over 6 years (2006-2011), when the power plant was set to work with full load. Features consist of hourly average ambient variables Temperature, Ambient Pressure, Relative Humidity and Exhaust Vacuum to predict the net hourly electrical energy output of the plant.</t>
   </si>
   <si>
-    <t>Folds5x2_pp.xlsx</t>
-  </si>
-  <si>
     <t>GREEND is an energy dataset containing power measurements collected from multiple households in Austria and Italy. It provides detailed energy profiles on a per device basis with a sampling rate of 1 Hz.</t>
   </si>
   <si>
@@ -236,9 +230,6 @@
   </si>
   <si>
     <t>We perform energy analysis using 12 different building shapes simulated in Ecotect. The buildings differ with respect to the glazing area, the glazing area distribution, and the orientation, amongst other parameters. We simulate various settings as functions of the afore-mentioned characteristics to obtain 768 building shapes. The dataset comprises 768 samples and 8 features, aiming to predict two real valued responses. It can also be used as a multi-class classification problem if the response is rounded to the nearest integer.</t>
-  </si>
-  <si>
-    <t>ENB2012_data.xlsx</t>
   </si>
   <si>
     <t>The data is collected from a smart small-scale steel industry in South Korea. The information gathered is from the DAEWOO Steel Co. Ltd in Gwangyang, South Korea. It produces several types of coils, steel plates, and iron plates. The information on electricity consumption is held in a cloud-based system. The information on energy consumption of the industry is stored on the website of the Korea Electric Power Corporation (pccs.kepco.go.kr), and the perspectives on daily, monthly, and annual data are calculated and shown.</t>
@@ -269,10 +260,6 @@
   </si>
   <si>
     <t>The PIRvision dataset contains occupancy detection data collected from a Synchronized Low-Energy Electronically-chopped Passive Infra-Red sensing node in residential and office environments. Each observation represents 4 seconds of recorded human activity within the sensor Field-of-View (FoV).</t>
-  </si>
-  <si>
-    <t>pirvision_office_dataset1.csv
-pirvision_office_dataset2.csv</t>
   </si>
   <si>
     <t>55+55</t>
@@ -310,9 +297,6 @@
   </si>
   <si>
     <t>50K</t>
-  </si>
-  <si>
-    <t>T1.csv</t>
   </si>
   <si>
     <t>The dataset contains eight attributes (or features) and two responses (or outcomes). The aim is to use the eight features to predict each of the two responses.</t>
@@ -602,6 +586,21 @@
   </si>
   <si>
     <t>pipe_thickness_loss_dataset.csv</t>
+  </si>
+  <si>
+    <t>Appliances Energy Prediction.csv</t>
+  </si>
+  <si>
+    <t>Combined Cycle Power Plant.csv</t>
+  </si>
+  <si>
+    <t>Energy_Efficiency.csv</t>
+  </si>
+  <si>
+    <t>pirvision_office_dataset1.csv</t>
+  </si>
+  <si>
+    <t>Wind Turbine Scada Dataset.csv</t>
   </si>
 </sst>
 </file>
@@ -666,7 +665,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -687,12 +686,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1244,7 +1237,7 @@
         <v>52</v>
       </c>
       <c r="E2" s="1">
-        <v>8417</v>
+        <v>4209</v>
       </c>
       <c r="F2" s="1">
         <v>385</v>
@@ -1275,7 +1268,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>59</v>
+        <v>171</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>6</v>
@@ -1295,13 +1288,13 @@
         <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>172</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E5" s="1">
         <v>9568</v>
@@ -1315,13 +1308,13 @@
         <v>9</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1331,13 +1324,13 @@
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1347,13 +1340,13 @@
         <v>13</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>66</v>
+        <v>173</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E8" s="1">
         <v>768</v>
@@ -1367,16 +1360,16 @@
         <v>15</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F9" s="1">
         <v>11</v>
@@ -1387,31 +1380,33 @@
         <v>17</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="F10" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="2"/>
+      <c r="B11" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="C11" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1421,19 +1416,19 @@
         <v>21</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>76</v>
+        <v>174</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>22</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
@@ -1441,13 +1436,13 @@
         <v>23</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E13" s="1">
         <v>1000</v>
@@ -1461,19 +1456,19 @@
         <v>33</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>34</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -1481,7 +1476,7 @@
         <v>35</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>36</v>
@@ -1495,16 +1490,16 @@
         <v>41</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>87</v>
+        <v>175</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F16" s="1">
         <v>5</v>
@@ -1515,13 +1510,13 @@
         <v>43</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>44</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E17" s="1">
         <v>768</v>
@@ -1532,16 +1527,16 @@
     </row>
     <row r="18" spans="1:6" ht="144" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E18" s="1">
         <v>1000</v>
@@ -1552,19 +1547,19 @@
     </row>
     <row r="19" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F19" s="1">
         <v>29</v>
@@ -1575,13 +1570,13 @@
         <v>46</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>45</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E20" s="1">
         <v>3650</v>
@@ -1591,364 +1586,364 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="1">
+        <v>5000</v>
+      </c>
+      <c r="F21" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B21" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D21" s="8" t="s">
+      <c r="E22" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="E21" s="9">
-        <v>5000</v>
-      </c>
-      <c r="F21" s="9">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
+      <c r="F22" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="D23" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E23" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F23" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="F22" s="9">
+      <c r="E24" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F24" s="1">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="E25" s="1">
+        <v>8737</v>
+      </c>
+      <c r="F25" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E26" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F26" s="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="144" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F27" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F28" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E29" s="1">
+        <v>500</v>
+      </c>
+      <c r="F29" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F30" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="D23" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E23" s="9">
+    <row r="31" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F31" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E33" s="1">
         <v>1000</v>
       </c>
-      <c r="F23" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D24" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="E24" s="9">
+      <c r="F33" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E34" s="1">
         <v>1000</v>
       </c>
-      <c r="F24" s="9">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="B25" s="8" t="s">
+      <c r="F34" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+    </row>
+    <row r="36" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+    </row>
+    <row r="37" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+    </row>
+    <row r="38" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C25" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="D25" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="E25" s="9">
-        <v>8737</v>
-      </c>
-      <c r="F25" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A26" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D26" s="8" t="s">
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+    </row>
+    <row r="39" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E26" s="9">
-        <v>1000</v>
-      </c>
-      <c r="F26" s="9">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="144" x14ac:dyDescent="0.3">
-      <c r="A27" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="E27" s="9">
-        <v>1000</v>
-      </c>
-      <c r="F27" s="9">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="E28" s="9">
-        <v>1000</v>
-      </c>
-      <c r="F28" s="9">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D29" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="E29" s="9">
-        <v>500</v>
-      </c>
-      <c r="F29" s="9">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="E30" s="9">
-        <v>1000</v>
-      </c>
-      <c r="F30" s="9">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="172.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="F31" s="9">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>164</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="B33" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D33" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="E33" s="9">
-        <v>1000</v>
-      </c>
-      <c r="F33" s="9">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A34" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="E34" s="9">
-        <v>1000</v>
-      </c>
-      <c r="F34" s="9">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="B35" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-    </row>
-    <row r="36" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="B36" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-    </row>
-    <row r="37" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A37" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-    </row>
-    <row r="38" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A38" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-    </row>
-    <row r="39" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A39" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>131</v>
-      </c>
       <c r="C39" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
+        <v>96</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="5"/>
@@ -2025,10 +2020,27 @@
     <hyperlink ref="C16" r:id="rId15" xr:uid="{C267BDF6-6DAA-4BA2-851A-D9DCD6829A3B}"/>
     <hyperlink ref="C17" r:id="rId16" xr:uid="{206B57A0-34C2-4D8E-A198-41735B03C771}"/>
     <hyperlink ref="C20" r:id="rId17" xr:uid="{0C83C8B7-B7B9-4FC9-8E4A-D3C6BD85EBF2}"/>
+    <hyperlink ref="C18" r:id="rId18" xr:uid="{406120BB-3953-43D0-9FD4-CD61DDBE00A7}"/>
+    <hyperlink ref="C19" r:id="rId19" xr:uid="{FB5FDC9C-2780-497C-B1D1-1385EBF112D8}"/>
+    <hyperlink ref="C21" r:id="rId20" xr:uid="{0311E65D-2F20-41D8-AB87-9DCA08DAC63F}"/>
+    <hyperlink ref="C22" r:id="rId21" xr:uid="{3E135099-BBA6-42A3-B0E2-EAB4653A5B3B}"/>
+    <hyperlink ref="C23" r:id="rId22" xr:uid="{B5C4FE78-8C3B-42E4-BB0A-B6C7A824CD7B}"/>
+    <hyperlink ref="C24" r:id="rId23" xr:uid="{ADDD48DB-1A1F-41AF-9F08-F298574E3161}"/>
+    <hyperlink ref="C25" r:id="rId24" xr:uid="{40B78C8C-5C0C-4AEC-9C7E-45477880B5CF}"/>
+    <hyperlink ref="C26" r:id="rId25" xr:uid="{3F35CD5E-E8BC-4AD9-87A6-113BB4698015}"/>
+    <hyperlink ref="C27" r:id="rId26" xr:uid="{85318783-700A-41E2-8B9B-8EE2D6E24C00}"/>
+    <hyperlink ref="C28" r:id="rId27" xr:uid="{263689D5-10A0-4199-BD14-A9632C6C37E6}"/>
+    <hyperlink ref="C29" r:id="rId28" xr:uid="{8F916FEB-9215-47AD-9BD0-B452051B88F6}"/>
+    <hyperlink ref="C30" r:id="rId29" xr:uid="{077FA9E7-B9E8-49AE-8276-62E8D4B2B82B}"/>
+    <hyperlink ref="C31" r:id="rId30" xr:uid="{0F02953C-A048-49F4-9577-5BE5BAB64BE8}"/>
+    <hyperlink ref="C32" r:id="rId31" xr:uid="{E2C8A966-A4C5-43C6-8FD6-212AFFC4222D}"/>
+    <hyperlink ref="C33" r:id="rId32" xr:uid="{1DA53EFB-A95C-4836-8F10-FC816ACD8D3D}"/>
+    <hyperlink ref="C34" r:id="rId33" xr:uid="{8CC3C032-73DE-40EC-89D9-2ACD4B097BCF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId34"/>
   <tableParts count="1">
-    <tablePart r:id="rId18"/>
+    <tablePart r:id="rId35"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>